<commit_message>
fix(#179): 补齐 RA SHA + F2/F3 标签
</commit_message>
<xml_diff>
--- a/docs/模型核验材料与数据申明清单_20261028.xlsx
+++ b/docs/模型核验材料与数据申明清单_20261028.xlsx
@@ -1118,7 +1118,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>成本核算脚本 cost.py</t>
+          <t>cost.py 与 submission.csv 一致性比对</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="B4" s="6" t="inlineStr">
         <is>
-          <t>逐图成本表</t>
+          <t>模型文件大小实测（解压后≤500MB）</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">

</xml_diff>